<commit_message>
Updates: grading, homework solutions, figures, new lecture notes and worksheets
</commit_message>
<xml_diff>
--- a/Grades/Grades.xlsx
+++ b/Grades/Grades.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
   <si>
     <t xml:space="preserve">First name</t>
   </si>
@@ -49,6 +49,9 @@
     <t xml:space="preserve">Midterm 1</t>
   </si>
   <si>
+    <t xml:space="preserve">Final Project Proposal</t>
+  </si>
+  <si>
     <t xml:space="preserve">Luka</t>
   </si>
   <si>
@@ -65,6 +68,9 @@
   </si>
   <si>
     <t xml:space="preserve">khewett@poets.whittier.edu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">--</t>
   </si>
   <si>
     <t xml:space="preserve">Gary</t>
@@ -211,8 +217,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultColWidth="8.51953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr defaultColWidth="8.5234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.3"/>
@@ -220,6 +226,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="17.95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -255,16 +262,19 @@
       <c r="K2" s="0" t="s">
         <v>8</v>
       </c>
+      <c r="L2" s="0" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F3" s="0" t="n">
         <f aca="false">12.5/17</f>
@@ -276,6 +286,14 @@
       <c r="H3" s="0" t="n">
         <v>0</v>
       </c>
+      <c r="I3" s="0" t="n">
+        <f aca="false">1</f>
+        <v>1</v>
+      </c>
+      <c r="J3" s="0" t="n">
+        <f aca="false">28/30</f>
+        <v>0.933333333333333</v>
+      </c>
       <c r="K3" s="0" t="n">
         <f aca="false">21/30</f>
         <v>0.7</v>
@@ -283,13 +301,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" s="0" t="n">
         <f aca="false">16/17</f>
@@ -301,20 +319,48 @@
       <c r="H4" s="0" t="n">
         <v>1</v>
       </c>
+      <c r="I4" s="0" t="n">
+        <f aca="false">1</f>
+        <v>1</v>
+      </c>
+      <c r="J4" s="0" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
       <c r="K4" s="0" t="n">
         <f aca="false">28.5/30</f>
         <v>0.95</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F5" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F6" s="0" t="n">
         <f aca="false">14/17</f>
@@ -326,6 +372,14 @@
       <c r="H6" s="0" t="n">
         <v>1</v>
       </c>
+      <c r="I6" s="0" t="n">
+        <f aca="false">1</f>
+        <v>1</v>
+      </c>
+      <c r="J6" s="0" t="n">
+        <f aca="false">27/30</f>
+        <v>0.9</v>
+      </c>
       <c r="K6" s="0" t="n">
         <f aca="false">27/30</f>
         <v>0.9</v>
@@ -333,13 +387,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F7" s="0" t="n">
         <f aca="false">11/17</f>
@@ -351,6 +405,14 @@
       <c r="H7" s="0" t="n">
         <v>1</v>
       </c>
+      <c r="I7" s="0" t="n">
+        <f aca="false">0.5</f>
+        <v>0.5</v>
+      </c>
+      <c r="J7" s="0" t="n">
+        <f aca="false">28/30</f>
+        <v>0.933333333333333</v>
+      </c>
       <c r="K7" s="0" t="n">
         <f aca="false">24/30</f>
         <v>0.8</v>
@@ -358,13 +420,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F8" s="0" t="n">
         <f aca="false">14/17</f>
@@ -376,6 +438,14 @@
       <c r="H8" s="0" t="n">
         <v>1</v>
       </c>
+      <c r="I8" s="0" t="n">
+        <f aca="false">0.67</f>
+        <v>0.67</v>
+      </c>
+      <c r="J8" s="0" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
       <c r="K8" s="0" t="n">
         <f aca="false">25.5/30</f>
         <v>0.85</v>
@@ -383,13 +453,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F9" s="0" t="n">
         <f aca="false">15/17</f>
@@ -401,6 +471,14 @@
       <c r="H9" s="0" t="n">
         <v>1</v>
       </c>
+      <c r="I9" s="0" t="n">
+        <f aca="false">0.67</f>
+        <v>0.67</v>
+      </c>
+      <c r="J9" s="0" t="n">
+        <f aca="false">25/30</f>
+        <v>0.833333333333333</v>
+      </c>
       <c r="K9" s="0" t="n">
         <f aca="false">26.5/30</f>
         <v>0.883333333333333</v>
@@ -408,13 +486,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F10" s="0" t="n">
         <f aca="false">14/17</f>
@@ -424,6 +502,14 @@
         <v>0</v>
       </c>
       <c r="H10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="0" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="0" t="n">
+        <f aca="false">0</f>
         <v>0</v>
       </c>
       <c r="K10" s="0" t="n">

</xml_diff>

<commit_message>
many figures, new lecture notes, downloaded homeworks
</commit_message>
<xml_diff>
--- a/Grades/Grades.xlsx
+++ b/Grades/Grades.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
   <si>
     <t xml:space="preserve">First name</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t xml:space="preserve">Final Project Proposal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homework 6</t>
   </si>
   <si>
     <t xml:space="preserve">Luka</t>
@@ -217,8 +220,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="8.5234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr defaultColWidth="8.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.3"/>
@@ -227,6 +230,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="17.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.3"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -265,16 +269,19 @@
       <c r="L2" s="0" t="s">
         <v>9</v>
       </c>
+      <c r="M2" s="0" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F3" s="0" t="n">
         <f aca="false">12.5/17</f>
@@ -298,16 +305,22 @@
         <f aca="false">21/30</f>
         <v>0.7</v>
       </c>
+      <c r="L3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="0" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F4" s="0" t="n">
         <f aca="false">16/17</f>
@@ -331,36 +344,43 @@
         <f aca="false">28.5/30</f>
         <v>0.95</v>
       </c>
+      <c r="L4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="0" t="n">
+        <f aca="false">9/10</f>
+        <v>0.9</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F5" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K5" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F6" s="0" t="n">
         <f aca="false">14/17</f>
@@ -384,16 +404,23 @@
         <f aca="false">27/30</f>
         <v>0.9</v>
       </c>
+      <c r="L6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="0" t="n">
+        <f aca="false">13/10</f>
+        <v>1.3</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F7" s="0" t="n">
         <f aca="false">11/17</f>
@@ -417,16 +444,23 @@
         <f aca="false">24/30</f>
         <v>0.8</v>
       </c>
+      <c r="L7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="0" t="n">
+        <f aca="false">13/10</f>
+        <v>1.3</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F8" s="0" t="n">
         <f aca="false">14/17</f>
@@ -450,16 +484,22 @@
         <f aca="false">25.5/30</f>
         <v>0.85</v>
       </c>
+      <c r="L8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="0" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F9" s="0" t="n">
         <f aca="false">15/17</f>
@@ -483,16 +523,23 @@
         <f aca="false">26.5/30</f>
         <v>0.883333333333333</v>
       </c>
+      <c r="L9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="0" t="n">
+        <f aca="false">10/10</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F10" s="0" t="n">
         <f aca="false">14/17</f>
@@ -515,6 +562,12 @@
       <c r="K10" s="0" t="n">
         <f aca="false">27/30</f>
         <v>0.9</v>
+      </c>
+      <c r="L10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
bit of a grade update
</commit_message>
<xml_diff>
--- a/Grades/Grades.xlsx
+++ b/Grades/Grades.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t xml:space="preserve">First name</t>
   </si>
@@ -53,6 +53,12 @@
   </si>
   <si>
     <t xml:space="preserve">Homework 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Midterm 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homework 7</t>
   </si>
   <si>
     <t xml:space="preserve">Luka</t>
@@ -220,8 +226,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
-  <sheetFormatPr defaultColWidth="8.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr defaultColWidth="8.5625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.3"/>
@@ -231,6 +237,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="17.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="11.09"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -272,16 +279,22 @@
       <c r="M2" s="0" t="s">
         <v>10</v>
       </c>
+      <c r="N2" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F3" s="0" t="n">
         <f aca="false">12.5/17</f>
@@ -314,13 +327,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F4" s="0" t="n">
         <f aca="false">16/17</f>
@@ -354,33 +367,33 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F5" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K5" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F6" s="0" t="n">
         <f aca="false">14/17</f>
@@ -414,13 +427,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F7" s="0" t="n">
         <f aca="false">11/17</f>
@@ -451,16 +464,20 @@
         <f aca="false">13/10</f>
         <v>1.3</v>
       </c>
+      <c r="O7" s="0" t="n">
+        <f aca="false">10/10</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F8" s="0" t="n">
         <f aca="false">14/17</f>
@@ -493,13 +510,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F9" s="0" t="n">
         <f aca="false">15/17</f>
@@ -533,23 +550,23 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F10" s="0" t="n">
         <f aca="false">14/17</f>
         <v>0.823529411764706</v>
       </c>
       <c r="G10" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" s="0" t="n">
         <f aca="false">0</f>

</xml_diff>

<commit_message>
grade update, old homeworks
</commit_message>
<xml_diff>
--- a/Grades/Grades.xlsx
+++ b/Grades/Grades.xlsx
@@ -230,7 +230,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P11"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.3"/>
@@ -648,12 +648,12 @@
         <v>1</v>
       </c>
       <c r="I10" s="0" t="n">
-        <f aca="false">0</f>
-        <v>0</v>
+        <f aca="false">1</f>
+        <v>1</v>
       </c>
       <c r="J10" s="0" t="n">
-        <f aca="false">0</f>
-        <v>0</v>
+        <f aca="false">24/30</f>
+        <v>0.8</v>
       </c>
       <c r="K10" s="0" t="n">
         <f aca="false">27/30</f>
@@ -663,7 +663,8 @@
         <v>1</v>
       </c>
       <c r="M10" s="0" t="n">
-        <v>0</v>
+        <f aca="false">10/10</f>
+        <v>1</v>
       </c>
       <c r="N10" s="0" t="n">
         <f aca="false">40/40</f>

</xml_diff>